<commit_message>
Add code to book tct with different payemnet method
</commit_message>
<xml_diff>
--- a/target/test-classes/BooKIngResistratinData.xlsx
+++ b/target/test-classes/BooKIngResistratinData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ravibhushan.Kumar\eclipse-workspace\Project_SAUDIA\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFE57D2-A67C-4D22-98F1-BF3BD298723B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC75D8DC-6C8F-435E-8E19-24EA8519B83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14040" xr2:uid="{95A23CBA-6176-416D-B3C6-85753400ABEE}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="117">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -111,9 +111,6 @@
     <t>md.nazir@quadlabs.com</t>
   </si>
   <si>
-    <t>8454963279</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 50-249 </t>
   </si>
   <si>
@@ -273,9 +270,6 @@
     <t>Prince</t>
   </si>
   <si>
-    <t>7896541236</t>
-  </si>
-  <si>
     <t>Department_Name</t>
   </si>
   <si>
@@ -360,18 +354,9 @@
     <t>Mr.</t>
   </si>
   <si>
-    <t>Ramesh</t>
-  </si>
-  <si>
-    <t>Mishra</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
-    <t>EMP012</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Administrator</t>
   </si>
   <si>
@@ -382,6 +367,18 @@
   </si>
   <si>
     <t>Password</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>Suresh</t>
+  </si>
+  <si>
+    <t>8789395155</t>
+  </si>
+  <si>
+    <t>EMP0124</t>
   </si>
 </sst>
 </file>
@@ -872,139 +869,139 @@
         <v>17</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="Y1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="AA1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AB1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="AD1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AE1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AG1" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="AH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AI1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="AM1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AQ1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="AR1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AS1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AT1" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="AU1" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AV1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="BC1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="BB1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BH1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="BJ1" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:62" x14ac:dyDescent="0.25">
@@ -1015,13 +1012,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>20</v>
@@ -1048,151 +1045,151 @@
         <v>26</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="1">
+        <v>4558975460</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="U2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="V2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="W2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="Y2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="AB2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AC2" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="AD2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AE2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AF2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AG2" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="AI2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AM2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="AN2" t="s">
         <v>78</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AO2" t="s">
         <v>79</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>80</v>
       </c>
       <c r="AP2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="AQ2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AR2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AS2" t="s">
         <v>83</v>
       </c>
-      <c r="AS2" t="s">
-        <v>85</v>
-      </c>
       <c r="AT2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AU2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="AV2" s="1" t="s">
+      <c r="AW2" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="AW2" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="AX2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AY2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AZ2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="BA2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BB2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AY2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AZ2" s="1" t="s">
+      <c r="BC2" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BA2" s="1" t="s">
+      <c r="BD2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="BE2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BF2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="BG2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="BB2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="BC2" s="1" t="s">
+      <c r="BH2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="BI2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="BD2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="BE2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="BF2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="BG2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BH2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="BI2" s="1" t="s">
-        <v>114</v>
-      </c>
       <c r="BJ2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:62" x14ac:dyDescent="0.25">

</xml_diff>